<commit_message>
Fatia 14A.1: as oito colunas de cada aba de detalhe sao conferidas
A automacao escreve oito valores; conferir seis deixava a possibilidade de
o oitavo cair sob um cabecalho de outro significado.

A oitava de Processos Fiscais foi decidida pelo PRODUTOR, e nao por voto
entre artefatos: o valor sai de div.processo-credito, revelado por um
botao cujo aria-label e "Expandir processo de credito". O codigo ja estava
certo; o PLANILHA MODELO.xlsx a chamava de Informacoes Complementares, que
e o rotulo do botao que ABRE o card. O modelo foi corrigido — duas celulas,
edicao ciruergica no zip, todas as outras partes byte a byte iguais.

A quinta ganhou um alias historico finito: o modelo trazia Dt. Vcto nesta
aba e Dt.Vcto. na de Debitos, discordando de si mesmo. A forma canonica e
a do codigo, e a antiga continua aceita para nao recusar planilha em uso.
Duas strings comprovadas, e nao uma regra de pontuacao.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PLANILHA MODELO.xlsx
+++ b/PLANILHA MODELO.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>CNPJ</t>
   </si>
@@ -89,6 +89,9 @@
   </si>
   <si>
     <t xml:space="preserve">Saldo Devedor </t>
+  </si>
+  <si>
+    <t>Processo de Crédito</t>
   </si>
 </sst>
 </file>
@@ -629,7 +632,7 @@
         <v>8</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>10</v>
@@ -638,7 +641,7 @@
         <v>15</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>